<commit_message>
Add pricing notes tab documenting every change and its source
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pricing Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15,12 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00;[Red]($#,##0.00)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +77,25 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -94,8 +113,23 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -146,13 +180,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -267,6 +315,24 @@
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:U122"/>
+  <dimension ref="A2:Q122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3881,4 +3947,453 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>PRICING NOTES — WHAT CHANGED AND WHY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="31" t="inlineStr">
+        <is>
+          <t>Every change below came off an actual Paychex invoice or from your 9/22 email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>CHANGED — 6 clients</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="n"/>
+      <c r="C4" s="33" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="33" t="n"/>
+      <c r="F4" s="33" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Your sheet</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Auction Time Pieces</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>154.1</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>75</v>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>Invoice shows Flex Select 79.10 plus Direct Deposit Premium Processing 75.00, charged every run.</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoice 7/30/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Onchain Strategies</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n">
+        <v>58</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>101</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>43</v>
+      </c>
+      <c r="E7" s="38" t="inlineStr">
+        <is>
+          <t>Base is Officer Only Payroll 65.00, not 58.00, plus Delivery 36.00 every run.</t>
+        </is>
+      </c>
+      <c r="F7" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoice 5/27/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Walters Mirrors</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>261.95</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>166.65</v>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>Paychex actually charges 502.15 a run on HR Pro. 261.95 is our price. Also bi-weekly not semi-monthly, 26 runs not 24, and 3 employees not 5.</t>
+        </is>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoices 9/2 + 9/14/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Complete Merchant Services</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n">
+        <v>70</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Not on Paychex. On Gusto at 100 a month, 2 employees, payroll only.</t>
+        </is>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>Your email 9/22/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>FRG Advisory</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n">
+        <v>70</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" s="37" t="n">
+        <v>-20</v>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>On Gusto at 50 a month, monthly.</t>
+        </is>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>Your email 9/22/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>Broadway 2000</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>400</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>No provider. Runs through IRS Treasury online, about 400 a year.</t>
+        </is>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>Your email 9/22/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>MATCHED YOUR SHEET EXACTLY — 3 clients</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="41" t="n"/>
+      <c r="D13" s="41" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>Wisdom by Woods</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>129.78</v>
+      </c>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="39" t="n"/>
+      <c r="E14" s="39" t="n"/>
+      <c r="F14" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoices 6/24 + 7/29/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>Backfin Logistics</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="C15" s="39" t="n"/>
+      <c r="D15" s="39" t="n"/>
+      <c r="E15" s="39" t="n"/>
+      <c r="F15" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoices 8/12, 8/26, 9/11/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>Spencer Thwaytes &amp; Co</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n">
+        <v>77</v>
+      </c>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="39" t="n"/>
+      <c r="E16" s="39" t="n"/>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>Paychex invoice 8/27/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED — 4 clients, your original figures kept</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="n"/>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="33" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>Upstate Logistics</t>
+        </is>
+      </c>
+      <c r="B19" s="36" t="n">
+        <v>78.56999999999999</v>
+      </c>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="39" t="n"/>
+      <c r="E19" s="39" t="inlineStr">
+        <is>
+          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+        </is>
+      </c>
+      <c r="F19" s="39" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>Tyree Advisory</t>
+        </is>
+      </c>
+      <c r="B20" s="36" t="n">
+        <v>71.92</v>
+      </c>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="39" t="n"/>
+      <c r="E20" s="39" t="inlineStr">
+        <is>
+          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+        </is>
+      </c>
+      <c r="F20" s="39" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>RJC Holdings</t>
+        </is>
+      </c>
+      <c r="B21" s="36" t="n">
+        <v>58</v>
+      </c>
+      <c r="C21" s="39" t="n"/>
+      <c r="D21" s="39" t="n"/>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+        </is>
+      </c>
+      <c r="F21" s="39" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="35" t="inlineStr">
+        <is>
+          <t>Kranz Motorcars</t>
+        </is>
+      </c>
+      <c r="B22" s="36" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="39" t="n"/>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
+          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+        </is>
+      </c>
+      <c r="F22" s="39" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>REMOVED — 5 clients with no current payroll billing</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="n"/>
+      <c r="C24" s="43" t="n"/>
+      <c r="D24" s="43" t="n"/>
+      <c r="E24" s="43" t="n"/>
+      <c r="F24" s="43" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>B333 Trading  ·  AJG Trading  ·  Kapstone Digital  ·  Atlas Opera  ·  North Star Works</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>WHAT IS NOT IN THESE NUMBERS</t>
+        </is>
+      </c>
+      <c r="B27" s="43" t="n"/>
+      <c r="C27" s="43" t="n"/>
+      <c r="D27" s="43" t="n"/>
+      <c r="E27" s="43" t="n"/>
+      <c r="F27" s="43" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>One-time setup fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Missing State ID and Missing Local ID penalties of 50 a month. Those stop once the registrations are filed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Year-end W-2 and 1099 charges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>401(k) fees. Those are priced separately.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mark access status instead of pricing-unconfirmed note
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0.00;[Red]($#,##0.00)"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,6 +93,10 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -200,7 +204,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -333,6 +337,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -678,8 +684,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:Q122"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
+  <dimension ref="A2:R122"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="14.28515625" customWidth="1" min="2" max="4"/>
@@ -691,6 +697,7 @@
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="15" max="16"/>
     <col width="18" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="38" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="2" ht="74.45" customHeight="1">
@@ -777,6 +784,11 @@
       <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>Total Current Annualized Billings (Excluding Year End/W2 Fees)</t>
+        </is>
+      </c>
+      <c r="R2" s="44" t="inlineStr">
+        <is>
+          <t>Access</t>
         </is>
       </c>
     </row>
@@ -974,6 +986,11 @@
         <f>M5</f>
         <v/>
       </c>
+      <c r="R5" s="45" t="inlineStr">
+        <is>
+          <t>No access — Paychex cannot link the account</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">
@@ -1038,6 +1055,11 @@
       <c r="Q6" s="23">
         <f>M6</f>
         <v/>
+      </c>
+      <c r="R6" s="45" t="inlineStr">
+        <is>
+          <t>No access — client has not granted it</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1670,11 +1692,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
-      <c r="B17" s="28" t="inlineStr">
-        <is>
-          <t>Shaded rows are estimates. Pricing on these four has moved around and was never confirmed.</t>
-        </is>
-      </c>
+      <c r="B17" s="28" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="1" t="n"/>
       <c r="E17" s="2" t="n"/>
@@ -1693,11 +1711,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t>Upstate Logistics  ·  Tyree Advisory  ·  RJC Holdings  ·  Kranz Motorcars</t>
-        </is>
-      </c>
+      <c r="B18" s="28" t="n"/>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="1" t="n"/>
       <c r="E18" s="2" t="n"/>
@@ -3956,7 +3970,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3980,6 +3994,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -4180,6 +4195,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="40" t="inlineStr">
         <is>
@@ -4246,10 +4262,11 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="32" t="inlineStr">
         <is>
-          <t>NOT CONFIRMED — 4 clients, your original figures kept</t>
+          <t>TOP FOUR — pricing still adjustable</t>
         </is>
       </c>
       <c r="B18" s="33" t="n"/>
@@ -4271,7 +4288,7 @@
       <c r="D19" s="39" t="n"/>
       <c r="E19" s="39" t="inlineStr">
         <is>
-          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+          <t>Access granted, invoice not received yet.</t>
         </is>
       </c>
       <c r="F19" s="39" t="n"/>
@@ -4289,7 +4306,7 @@
       <c r="D20" s="39" t="n"/>
       <c r="E20" s="39" t="inlineStr">
         <is>
-          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+          <t>Access granted, invoice not received yet.</t>
         </is>
       </c>
       <c r="F20" s="39" t="n"/>
@@ -4307,7 +4324,7 @@
       <c r="D21" s="39" t="n"/>
       <c r="E21" s="39" t="inlineStr">
         <is>
-          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+          <t>No access. Paychex cannot link the account.</t>
         </is>
       </c>
       <c r="F21" s="39" t="n"/>
@@ -4325,7 +4342,7 @@
       <c r="D22" s="39" t="n"/>
       <c r="E22" s="39" t="inlineStr">
         <is>
-          <t>No invoice received. Pricing has moved around and was never confirmed.</t>
+          <t>No access. Client has not granted it.</t>
         </is>
       </c>
       <c r="F22" s="39" t="n"/>

</xml_diff>

<commit_message>
Remove shading from the top four rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
@@ -204,7 +204,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -339,6 +339,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -685,7 +689,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:R122"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="14.28515625" customWidth="1" min="2" max="4"/>
@@ -793,196 +797,196 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="n">
+      <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Robert</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Tupe</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>Upstate Logistics Group LLC</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>33-4154077</t>
         </is>
       </c>
-      <c r="G3" s="16" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>2107 Goldfinch Blvd</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Princeton, NJ 08540</t>
         </is>
       </c>
-      <c r="I3" s="18" t="n">
+      <c r="I3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="18" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Biweekly</t>
         </is>
       </c>
-      <c r="K3" s="19" t="n">
+      <c r="K3" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="L3" s="20" t="n">
+      <c r="L3" s="24" t="n">
         <v>78.56999999999999</v>
       </c>
-      <c r="M3" s="20">
+      <c r="M3" s="24">
         <f>K3*L3</f>
         <v/>
       </c>
-      <c r="N3" s="21" t="n"/>
-      <c r="O3" s="22" t="n"/>
-      <c r="P3" s="22" t="n"/>
-      <c r="Q3" s="23">
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="25" t="n"/>
+      <c r="P3" s="25" t="n"/>
+      <c r="Q3" s="26">
         <f>M3</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Ty</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Tyree</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Tyree Advisory Group LLC</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>42-1951214</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>106 W Dorothys Way</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Lincoln University, PA 19352</t>
         </is>
       </c>
-      <c r="I4" s="18" t="n">
+      <c r="I4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="K4" s="19" t="n">
+      <c r="K4" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L4" s="20" t="n">
+      <c r="L4" s="24" t="n">
         <v>71.92</v>
       </c>
-      <c r="M4" s="20">
+      <c r="M4" s="24">
         <f>K4*L4</f>
         <v/>
       </c>
-      <c r="N4" s="21" t="n"/>
-      <c r="O4" s="22" t="n"/>
-      <c r="P4" s="22" t="n"/>
-      <c r="Q4" s="23">
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="25" t="n"/>
+      <c r="P4" s="25" t="n"/>
+      <c r="Q4" s="26">
         <f>M4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ricardo </t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>De'Carvalho</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>RJC Holdings</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>86-2385686</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>6278 North Federal Highway</t>
         </is>
       </c>
-      <c r="H5" s="16" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Fort Lauderdale, FL 33308</t>
         </is>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="18" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K5" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="L5" s="24" t="n">
         <v>58</v>
       </c>
-      <c r="M5" s="20">
+      <c r="M5" s="24">
         <f>K5*L5</f>
         <v/>
       </c>
-      <c r="N5" s="21" t="n"/>
-      <c r="O5" s="22" t="n"/>
-      <c r="P5" s="22" t="n"/>
-      <c r="Q5" s="23">
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="25" t="n"/>
+      <c r="P5" s="25" t="n"/>
+      <c r="Q5" s="26">
         <f>M5</f>
         <v/>
       </c>
@@ -993,66 +997,66 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Heather</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Kranz</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Existing</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Kranz Motorcars LLC</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>39-2155930</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>432 S Walnut St</t>
         </is>
       </c>
-      <c r="H6" s="16" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Kennett Square, PA 19348</t>
         </is>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="18" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Weekly</t>
         </is>
       </c>
-      <c r="K6" s="19" t="n">
+      <c r="K6" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="L6" s="20" t="n">
+      <c r="L6" s="24" t="n">
         <v>59.5</v>
       </c>
-      <c r="M6" s="20">
+      <c r="M6" s="24">
         <f>K6*L6</f>
         <v/>
       </c>
-      <c r="N6" s="21" t="n"/>
-      <c r="O6" s="22" t="n"/>
-      <c r="P6" s="22" t="n"/>
-      <c r="Q6" s="23">
+      <c r="N6" s="6" t="n"/>
+      <c r="O6" s="25" t="n"/>
+      <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="26">
         <f>M6</f>
         <v/>
       </c>
@@ -3970,7 +3974,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -3994,7 +3998,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -4195,7 +4198,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="40" t="inlineStr">
         <is>
@@ -4262,7 +4264,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Strip empty and duplicate columns and dead rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:R122"/>
+  <dimension ref="A1:O122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -699,11 +699,12 @@
     <col width="14.28515625" customWidth="1" min="10" max="10"/>
     <col width="15" bestFit="1" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="15" customWidth="1" min="15" max="16"/>
+    <col width="38" customWidth="1" min="15" max="16"/>
     <col width="18" bestFit="1" customWidth="1" min="17" max="17"/>
     <col width="38" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="74.45" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
@@ -775,22 +776,7 @@
           <t>401K Plan</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
-        <is>
-          <t>401K Fees</t>
-        </is>
-      </c>
-      <c r="P2" s="7" t="inlineStr">
-        <is>
-          <t>Other CY Fees</t>
-        </is>
-      </c>
-      <c r="Q2" s="7" t="inlineStr">
-        <is>
-          <t>Total Current Annualized Billings (Excluding Year End/W2 Fees)</t>
-        </is>
-      </c>
-      <c r="R2" s="44" t="inlineStr">
+      <c r="O2" s="44" t="inlineStr">
         <is>
           <t>Access</t>
         </is>
@@ -854,12 +840,6 @@
         <v/>
       </c>
       <c r="N3" s="6" t="n"/>
-      <c r="O3" s="25" t="n"/>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="26">
-        <f>M3</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -919,12 +899,6 @@
         <v/>
       </c>
       <c r="N4" s="6" t="n"/>
-      <c r="O4" s="25" t="n"/>
-      <c r="P4" s="25" t="n"/>
-      <c r="Q4" s="26">
-        <f>M4</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -984,13 +958,7 @@
         <v/>
       </c>
       <c r="N5" s="6" t="n"/>
-      <c r="O5" s="25" t="n"/>
-      <c r="P5" s="25" t="n"/>
-      <c r="Q5" s="26">
-        <f>M5</f>
-        <v/>
-      </c>
-      <c r="R5" s="45" t="inlineStr">
+      <c r="O5" s="45" t="inlineStr">
         <is>
           <t>No access — Paychex cannot link the account</t>
         </is>
@@ -1054,13 +1022,7 @@
         <v/>
       </c>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="25" t="n"/>
-      <c r="P6" s="25" t="n"/>
-      <c r="Q6" s="26">
-        <f>M6</f>
-        <v/>
-      </c>
-      <c r="R6" s="45" t="inlineStr">
+      <c r="O6" s="45" t="inlineStr">
         <is>
           <t>No access — client has not granted it</t>
         </is>
@@ -1124,12 +1086,6 @@
         <v/>
       </c>
       <c r="N7" s="6" t="n"/>
-      <c r="O7" s="25" t="n"/>
-      <c r="P7" s="25" t="n"/>
-      <c r="Q7" s="26">
-        <f>M7</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1189,12 +1145,6 @@
         <v/>
       </c>
       <c r="N8" s="6" t="n"/>
-      <c r="O8" s="25" t="n"/>
-      <c r="P8" s="25" t="n"/>
-      <c r="Q8" s="26">
-        <f>M8</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1258,12 +1208,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O9" s="25" t="n"/>
-      <c r="P9" s="25" t="n"/>
-      <c r="Q9" s="26">
-        <f>M9</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1323,12 +1267,6 @@
         <v/>
       </c>
       <c r="N10" s="6" t="n"/>
-      <c r="O10" s="25" t="n"/>
-      <c r="P10" s="25" t="n"/>
-      <c r="Q10" s="26">
-        <f>M10</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1392,12 +1330,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O11" s="25" t="n"/>
-      <c r="P11" s="25" t="n"/>
-      <c r="Q11" s="26">
-        <f>M11</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1461,12 +1393,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O12" s="25" t="n"/>
-      <c r="P12" s="25" t="n"/>
-      <c r="Q12" s="26">
-        <f>M12</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1530,12 +1456,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O13" s="4" t="n"/>
-      <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="26">
-        <f>M13</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1599,12 +1519,6 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="O14" s="4" t="n"/>
-      <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="26">
-        <f>M14</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1667,12 +1581,6 @@
         <is>
           <t>Yes</t>
         </is>
-      </c>
-      <c r="O15" s="4" t="n"/>
-      <c r="P15" s="4" t="n"/>
-      <c r="Q15" s="26">
-        <f>M15</f>
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -1690,9 +1598,6 @@
       <c r="L16" s="27" t="n"/>
       <c r="M16" s="6" t="n"/>
       <c r="N16" s="6" t="n"/>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -1709,9 +1614,6 @@
       <c r="L17" s="27" t="n"/>
       <c r="M17" s="6" t="n"/>
       <c r="N17" s="6" t="n"/>
-      <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -1728,9 +1630,6 @@
       <c r="L18" s="27" t="n"/>
       <c r="M18" s="6" t="n"/>
       <c r="N18" s="6" t="n"/>
-      <c r="O18" s="4" t="n"/>
-      <c r="P18" s="4" t="n"/>
-      <c r="Q18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -1747,9 +1646,6 @@
       <c r="L19" s="27" t="n"/>
       <c r="M19" s="6" t="n"/>
       <c r="N19" s="6" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -1766,14 +1662,9 @@
       <c r="L20" s="27" t="n"/>
       <c r="M20" s="6" t="n"/>
       <c r="N20" s="6" t="n"/>
-      <c r="O20" s="4" t="n"/>
-      <c r="P20" s="4" t="n"/>
-      <c r="Q20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>19</v>
-      </c>
+      <c r="A21" s="1" t="n"/>
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="1" t="n"/>
@@ -1787,14 +1678,9 @@
       <c r="L21" s="27" t="n"/>
       <c r="M21" s="6" t="n"/>
       <c r="N21" s="6" t="n"/>
-      <c r="O21" s="4" t="n"/>
-      <c r="P21" s="4" t="n"/>
-      <c r="Q21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>20</v>
-      </c>
+      <c r="A22" s="1" t="n"/>
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="1" t="n"/>
@@ -1808,14 +1694,9 @@
       <c r="L22" s="27" t="n"/>
       <c r="M22" s="6" t="n"/>
       <c r="N22" s="6" t="n"/>
-      <c r="O22" s="4" t="n"/>
-      <c r="P22" s="4" t="n"/>
-      <c r="Q22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>21</v>
-      </c>
+      <c r="A23" s="1" t="n"/>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="1" t="n"/>
@@ -1829,14 +1710,9 @@
       <c r="L23" s="27" t="n"/>
       <c r="M23" s="6" t="n"/>
       <c r="N23" s="6" t="n"/>
-      <c r="O23" s="4" t="n"/>
-      <c r="P23" s="4" t="n"/>
-      <c r="Q23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>22</v>
-      </c>
+      <c r="A24" s="1" t="n"/>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="1" t="n"/>
@@ -1850,14 +1726,9 @@
       <c r="L24" s="27" t="n"/>
       <c r="M24" s="6" t="n"/>
       <c r="N24" s="6" t="n"/>
-      <c r="O24" s="4" t="n"/>
-      <c r="P24" s="4" t="n"/>
-      <c r="Q24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>23</v>
-      </c>
+      <c r="A25" s="1" t="n"/>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="1" t="n"/>
@@ -1871,14 +1742,9 @@
       <c r="L25" s="27" t="n"/>
       <c r="M25" s="6" t="n"/>
       <c r="N25" s="6" t="n"/>
-      <c r="O25" s="4" t="n"/>
-      <c r="P25" s="4" t="n"/>
-      <c r="Q25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>24</v>
-      </c>
+      <c r="A26" s="1" t="n"/>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="1" t="n"/>
@@ -1892,14 +1758,9 @@
       <c r="L26" s="27" t="n"/>
       <c r="M26" s="6" t="n"/>
       <c r="N26" s="6" t="n"/>
-      <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
-      <c r="Q26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>25</v>
-      </c>
+      <c r="A27" s="1" t="n"/>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="1" t="n"/>
@@ -1913,14 +1774,9 @@
       <c r="L27" s="27" t="n"/>
       <c r="M27" s="6" t="n"/>
       <c r="N27" s="6" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>26</v>
-      </c>
+      <c r="A28" s="1" t="n"/>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="1" t="n"/>
       <c r="D28" s="1" t="n"/>
@@ -1934,9 +1790,6 @@
       <c r="L28" s="27" t="n"/>
       <c r="M28" s="6" t="n"/>
       <c r="N28" s="6" t="n"/>
-      <c r="O28" s="4" t="n"/>
-      <c r="P28" s="4" t="n"/>
-      <c r="Q28" s="5" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A29" s="1" t="n">
@@ -1962,14 +1815,9 @@
         <v/>
       </c>
       <c r="N29" s="6" t="n"/>
-      <c r="O29" s="4" t="n"/>
-      <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="5" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" thickTop="1">
-      <c r="A30" s="1" t="n">
-        <v>28</v>
-      </c>
+      <c r="A30" s="1" t="n"/>
       <c r="B30" s="1" t="n"/>
       <c r="C30" s="1" t="n"/>
       <c r="D30" s="1" t="n"/>
@@ -1983,9 +1831,6 @@
       <c r="L30" s="29" t="n"/>
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="6" t="n"/>
-      <c r="O30" s="4" t="n"/>
-      <c r="P30" s="4" t="n"/>
-      <c r="Q30" s="5" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" thickBot="1">
       <c r="A31" s="1" t="n">
@@ -2011,14 +1856,9 @@
         <v/>
       </c>
       <c r="N31" s="6" t="n"/>
-      <c r="O31" s="4" t="n"/>
-      <c r="P31" s="4" t="n"/>
-      <c r="Q31" s="5" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" thickTop="1">
-      <c r="A32" s="1" t="n">
-        <v>30</v>
-      </c>
+      <c r="A32" s="1" t="n"/>
       <c r="B32" s="1" t="n"/>
       <c r="C32" s="1" t="n"/>
       <c r="D32" s="1" t="n"/>
@@ -2032,14 +1872,9 @@
       <c r="L32" s="27" t="n"/>
       <c r="M32" s="11" t="n"/>
       <c r="N32" s="6" t="n"/>
-      <c r="O32" s="4" t="n"/>
-      <c r="P32" s="4" t="n"/>
-      <c r="Q32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>31</v>
-      </c>
+      <c r="A33" s="1" t="n"/>
       <c r="B33" s="1" t="n"/>
       <c r="C33" s="1" t="n"/>
       <c r="D33" s="1" t="n"/>
@@ -2053,14 +1888,9 @@
       <c r="L33" s="27" t="n"/>
       <c r="M33" s="6" t="n"/>
       <c r="N33" s="6" t="n"/>
-      <c r="O33" s="4" t="n"/>
-      <c r="P33" s="4" t="n"/>
-      <c r="Q33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>32</v>
-      </c>
+      <c r="A34" s="1" t="n"/>
       <c r="B34" s="1" t="n"/>
       <c r="C34" s="1" t="n"/>
       <c r="D34" s="1" t="n"/>
@@ -2074,14 +1904,9 @@
       <c r="L34" s="27" t="n"/>
       <c r="M34" s="6" t="n"/>
       <c r="N34" s="6" t="n"/>
-      <c r="O34" s="4" t="n"/>
-      <c r="P34" s="4" t="n"/>
-      <c r="Q34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>33</v>
-      </c>
+      <c r="A35" s="1" t="n"/>
       <c r="B35" s="1" t="n"/>
       <c r="C35" s="1" t="n"/>
       <c r="D35" s="1" t="n"/>
@@ -2095,14 +1920,9 @@
       <c r="L35" s="27" t="n"/>
       <c r="M35" s="6" t="n"/>
       <c r="N35" s="6" t="n"/>
-      <c r="O35" s="4" t="n"/>
-      <c r="P35" s="4" t="n"/>
-      <c r="Q35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>34</v>
-      </c>
+      <c r="A36" s="1" t="n"/>
       <c r="B36" s="1" t="n"/>
       <c r="C36" s="1" t="n"/>
       <c r="D36" s="1" t="n"/>
@@ -2116,14 +1936,9 @@
       <c r="L36" s="27" t="n"/>
       <c r="M36" s="6" t="n"/>
       <c r="N36" s="6" t="n"/>
-      <c r="O36" s="4" t="n"/>
-      <c r="P36" s="4" t="n"/>
-      <c r="Q36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
-      </c>
+      <c r="A37" s="1" t="n"/>
       <c r="B37" s="1" t="n"/>
       <c r="C37" s="1" t="n"/>
       <c r="D37" s="1" t="n"/>
@@ -2137,14 +1952,9 @@
       <c r="L37" s="27" t="n"/>
       <c r="M37" s="6" t="n"/>
       <c r="N37" s="6" t="n"/>
-      <c r="O37" s="4" t="n"/>
-      <c r="P37" s="4" t="n"/>
-      <c r="Q37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>36</v>
-      </c>
+      <c r="A38" s="1" t="n"/>
       <c r="B38" s="1" t="n"/>
       <c r="C38" s="1" t="n"/>
       <c r="D38" s="1" t="n"/>
@@ -2158,14 +1968,9 @@
       <c r="L38" s="27" t="n"/>
       <c r="M38" s="6" t="n"/>
       <c r="N38" s="6" t="n"/>
-      <c r="O38" s="4" t="n"/>
-      <c r="P38" s="4" t="n"/>
-      <c r="Q38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>37</v>
-      </c>
+      <c r="A39" s="1" t="n"/>
       <c r="B39" s="1" t="n"/>
       <c r="C39" s="1" t="n"/>
       <c r="D39" s="1" t="n"/>
@@ -2179,14 +1984,9 @@
       <c r="L39" s="27" t="n"/>
       <c r="M39" s="6" t="n"/>
       <c r="N39" s="6" t="n"/>
-      <c r="O39" s="4" t="n"/>
-      <c r="P39" s="4" t="n"/>
-      <c r="Q39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>38</v>
-      </c>
+      <c r="A40" s="1" t="n"/>
       <c r="B40" s="1" t="n"/>
       <c r="C40" s="1" t="n"/>
       <c r="D40" s="1" t="n"/>
@@ -2200,14 +2000,9 @@
       <c r="L40" s="27" t="n"/>
       <c r="M40" s="6" t="n"/>
       <c r="N40" s="6" t="n"/>
-      <c r="O40" s="4" t="n"/>
-      <c r="P40" s="4" t="n"/>
-      <c r="Q40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>39</v>
-      </c>
+      <c r="A41" s="1" t="n"/>
       <c r="B41" s="1" t="n"/>
       <c r="C41" s="1" t="n"/>
       <c r="D41" s="1" t="n"/>
@@ -2221,14 +2016,9 @@
       <c r="L41" s="27" t="n"/>
       <c r="M41" s="6" t="n"/>
       <c r="N41" s="6" t="n"/>
-      <c r="O41" s="4" t="n"/>
-      <c r="P41" s="4" t="n"/>
-      <c r="Q41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>40</v>
-      </c>
+      <c r="A42" s="1" t="n"/>
       <c r="B42" s="1" t="n"/>
       <c r="C42" s="1" t="n"/>
       <c r="D42" s="1" t="n"/>
@@ -2242,14 +2032,9 @@
       <c r="L42" s="27" t="n"/>
       <c r="M42" s="6" t="n"/>
       <c r="N42" s="6" t="n"/>
-      <c r="O42" s="4" t="n"/>
-      <c r="P42" s="4" t="n"/>
-      <c r="Q42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>41</v>
-      </c>
+      <c r="A43" s="1" t="n"/>
       <c r="B43" s="1" t="n"/>
       <c r="C43" s="1" t="n"/>
       <c r="D43" s="1" t="n"/>
@@ -2263,14 +2048,9 @@
       <c r="L43" s="27" t="n"/>
       <c r="M43" s="6" t="n"/>
       <c r="N43" s="6" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42</v>
-      </c>
+      <c r="A44" s="1" t="n"/>
       <c r="B44" s="1" t="n"/>
       <c r="C44" s="1" t="n"/>
       <c r="D44" s="1" t="n"/>
@@ -2284,14 +2064,9 @@
       <c r="L44" s="27" t="n"/>
       <c r="M44" s="6" t="n"/>
       <c r="N44" s="6" t="n"/>
-      <c r="O44" s="4" t="n"/>
-      <c r="P44" s="4" t="n"/>
-      <c r="Q44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>43</v>
-      </c>
+      <c r="A45" s="1" t="n"/>
       <c r="B45" s="1" t="n"/>
       <c r="C45" s="1" t="n"/>
       <c r="D45" s="1" t="n"/>
@@ -2305,14 +2080,9 @@
       <c r="L45" s="4" t="n"/>
       <c r="M45" s="6" t="n"/>
       <c r="N45" s="6" t="n"/>
-      <c r="O45" s="4" t="n"/>
-      <c r="P45" s="4" t="n"/>
-      <c r="Q45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>44</v>
-      </c>
+      <c r="A46" s="1" t="n"/>
       <c r="B46" s="1" t="n"/>
       <c r="C46" s="1" t="n"/>
       <c r="D46" s="1" t="n"/>
@@ -2326,14 +2096,9 @@
       <c r="L46" s="4" t="n"/>
       <c r="M46" s="6" t="n"/>
       <c r="N46" s="6" t="n"/>
-      <c r="O46" s="4" t="n"/>
-      <c r="P46" s="4" t="n"/>
-      <c r="Q46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>45</v>
-      </c>
+      <c r="A47" s="1" t="n"/>
       <c r="B47" s="1" t="n"/>
       <c r="C47" s="1" t="n"/>
       <c r="D47" s="1" t="n"/>
@@ -2347,14 +2112,9 @@
       <c r="L47" s="4" t="n"/>
       <c r="M47" s="6" t="n"/>
       <c r="N47" s="6" t="n"/>
-      <c r="O47" s="4" t="n"/>
-      <c r="P47" s="4" t="n"/>
-      <c r="Q47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>46</v>
-      </c>
+      <c r="A48" s="1" t="n"/>
       <c r="B48" s="1" t="n"/>
       <c r="C48" s="1" t="n"/>
       <c r="D48" s="1" t="n"/>
@@ -2368,14 +2128,9 @@
       <c r="L48" s="4" t="n"/>
       <c r="M48" s="6" t="n"/>
       <c r="N48" s="6" t="n"/>
-      <c r="O48" s="4" t="n"/>
-      <c r="P48" s="4" t="n"/>
-      <c r="Q48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>47</v>
-      </c>
+      <c r="A49" s="1" t="n"/>
       <c r="B49" s="1" t="n"/>
       <c r="C49" s="1" t="n"/>
       <c r="D49" s="1" t="n"/>
@@ -2389,14 +2144,9 @@
       <c r="L49" s="4" t="n"/>
       <c r="M49" s="6" t="n"/>
       <c r="N49" s="6" t="n"/>
-      <c r="O49" s="4" t="n"/>
-      <c r="P49" s="4" t="n"/>
-      <c r="Q49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>48</v>
-      </c>
+      <c r="A50" s="1" t="n"/>
       <c r="B50" s="1" t="n"/>
       <c r="C50" s="1" t="n"/>
       <c r="D50" s="1" t="n"/>
@@ -2410,14 +2160,9 @@
       <c r="L50" s="4" t="n"/>
       <c r="M50" s="6" t="n"/>
       <c r="N50" s="6" t="n"/>
-      <c r="O50" s="4" t="n"/>
-      <c r="P50" s="4" t="n"/>
-      <c r="Q50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>49</v>
-      </c>
+      <c r="A51" s="1" t="n"/>
       <c r="B51" s="1" t="n"/>
       <c r="C51" s="1" t="n"/>
       <c r="D51" s="1" t="n"/>
@@ -2431,14 +2176,9 @@
       <c r="L51" s="4" t="n"/>
       <c r="M51" s="6" t="n"/>
       <c r="N51" s="6" t="n"/>
-      <c r="O51" s="4" t="n"/>
-      <c r="P51" s="4" t="n"/>
-      <c r="Q51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>50</v>
-      </c>
+      <c r="A52" s="1" t="n"/>
       <c r="B52" s="1" t="n"/>
       <c r="C52" s="1" t="n"/>
       <c r="D52" s="1" t="n"/>
@@ -2452,14 +2192,9 @@
       <c r="L52" s="4" t="n"/>
       <c r="M52" s="6" t="n"/>
       <c r="N52" s="6" t="n"/>
-      <c r="O52" s="4" t="n"/>
-      <c r="P52" s="4" t="n"/>
-      <c r="Q52" s="5" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>51</v>
-      </c>
+      <c r="A53" s="1" t="n"/>
       <c r="B53" s="1" t="n"/>
       <c r="C53" s="1" t="n"/>
       <c r="D53" s="1" t="n"/>
@@ -2473,14 +2208,9 @@
       <c r="L53" s="4" t="n"/>
       <c r="M53" s="6" t="n"/>
       <c r="N53" s="6" t="n"/>
-      <c r="O53" s="4" t="n"/>
-      <c r="P53" s="4" t="n"/>
-      <c r="Q53" s="5" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>52</v>
-      </c>
+      <c r="A54" s="1" t="n"/>
       <c r="B54" s="1" t="n"/>
       <c r="C54" s="1" t="n"/>
       <c r="D54" s="1" t="n"/>
@@ -2494,14 +2224,9 @@
       <c r="L54" s="4" t="n"/>
       <c r="M54" s="6" t="n"/>
       <c r="N54" s="6" t="n"/>
-      <c r="O54" s="4" t="n"/>
-      <c r="P54" s="4" t="n"/>
-      <c r="Q54" s="5" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>53</v>
-      </c>
+      <c r="A55" s="1" t="n"/>
       <c r="B55" s="1" t="n"/>
       <c r="C55" s="1" t="n"/>
       <c r="D55" s="1" t="n"/>
@@ -2515,14 +2240,9 @@
       <c r="L55" s="4" t="n"/>
       <c r="M55" s="6" t="n"/>
       <c r="N55" s="6" t="n"/>
-      <c r="O55" s="4" t="n"/>
-      <c r="P55" s="4" t="n"/>
-      <c r="Q55" s="5" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>54</v>
-      </c>
+      <c r="A56" s="1" t="n"/>
       <c r="B56" s="1" t="n"/>
       <c r="C56" s="1" t="n"/>
       <c r="D56" s="1" t="n"/>
@@ -2536,14 +2256,9 @@
       <c r="L56" s="4" t="n"/>
       <c r="M56" s="6" t="n"/>
       <c r="N56" s="6" t="n"/>
-      <c r="O56" s="4" t="n"/>
-      <c r="P56" s="4" t="n"/>
-      <c r="Q56" s="5" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>55</v>
-      </c>
+      <c r="A57" s="1" t="n"/>
       <c r="B57" s="1" t="n"/>
       <c r="C57" s="1" t="n"/>
       <c r="D57" s="1" t="n"/>
@@ -2557,14 +2272,9 @@
       <c r="L57" s="4" t="n"/>
       <c r="M57" s="6" t="n"/>
       <c r="N57" s="6" t="n"/>
-      <c r="O57" s="4" t="n"/>
-      <c r="P57" s="4" t="n"/>
-      <c r="Q57" s="5" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>56</v>
-      </c>
+      <c r="A58" s="1" t="n"/>
       <c r="B58" s="1" t="n"/>
       <c r="C58" s="1" t="n"/>
       <c r="D58" s="1" t="n"/>
@@ -2578,14 +2288,9 @@
       <c r="L58" s="4" t="n"/>
       <c r="M58" s="6" t="n"/>
       <c r="N58" s="6" t="n"/>
-      <c r="O58" s="4" t="n"/>
-      <c r="P58" s="4" t="n"/>
-      <c r="Q58" s="5" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>57</v>
-      </c>
+      <c r="A59" s="1" t="n"/>
       <c r="B59" s="1" t="n"/>
       <c r="C59" s="1" t="n"/>
       <c r="D59" s="1" t="n"/>
@@ -2599,14 +2304,9 @@
       <c r="L59" s="4" t="n"/>
       <c r="M59" s="6" t="n"/>
       <c r="N59" s="6" t="n"/>
-      <c r="O59" s="4" t="n"/>
-      <c r="P59" s="4" t="n"/>
-      <c r="Q59" s="5" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>58</v>
-      </c>
+      <c r="A60" s="1" t="n"/>
       <c r="B60" s="1" t="n"/>
       <c r="C60" s="1" t="n"/>
       <c r="D60" s="1" t="n"/>
@@ -2620,14 +2320,9 @@
       <c r="L60" s="4" t="n"/>
       <c r="M60" s="6" t="n"/>
       <c r="N60" s="6" t="n"/>
-      <c r="O60" s="4" t="n"/>
-      <c r="P60" s="4" t="n"/>
-      <c r="Q60" s="5" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>59</v>
-      </c>
+      <c r="A61" s="1" t="n"/>
       <c r="B61" s="1" t="n"/>
       <c r="C61" s="1" t="n"/>
       <c r="D61" s="1" t="n"/>
@@ -2641,14 +2336,9 @@
       <c r="L61" s="4" t="n"/>
       <c r="M61" s="6" t="n"/>
       <c r="N61" s="6" t="n"/>
-      <c r="O61" s="4" t="n"/>
-      <c r="P61" s="4" t="n"/>
-      <c r="Q61" s="5" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>60</v>
-      </c>
+      <c r="A62" s="1" t="n"/>
       <c r="B62" s="1" t="n"/>
       <c r="C62" s="1" t="n"/>
       <c r="D62" s="1" t="n"/>
@@ -2662,14 +2352,9 @@
       <c r="L62" s="4" t="n"/>
       <c r="M62" s="6" t="n"/>
       <c r="N62" s="6" t="n"/>
-      <c r="O62" s="4" t="n"/>
-      <c r="P62" s="4" t="n"/>
-      <c r="Q62" s="5" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>61</v>
-      </c>
+      <c r="A63" s="1" t="n"/>
       <c r="B63" s="1" t="n"/>
       <c r="C63" s="1" t="n"/>
       <c r="D63" s="1" t="n"/>
@@ -2683,14 +2368,9 @@
       <c r="L63" s="4" t="n"/>
       <c r="M63" s="6" t="n"/>
       <c r="N63" s="6" t="n"/>
-      <c r="O63" s="4" t="n"/>
-      <c r="P63" s="4" t="n"/>
-      <c r="Q63" s="5" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>62</v>
-      </c>
+      <c r="A64" s="1" t="n"/>
       <c r="B64" s="1" t="n"/>
       <c r="C64" s="1" t="n"/>
       <c r="D64" s="1" t="n"/>
@@ -2704,14 +2384,9 @@
       <c r="L64" s="4" t="n"/>
       <c r="M64" s="6" t="n"/>
       <c r="N64" s="6" t="n"/>
-      <c r="O64" s="4" t="n"/>
-      <c r="P64" s="4" t="n"/>
-      <c r="Q64" s="5" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>63</v>
-      </c>
+      <c r="A65" s="1" t="n"/>
       <c r="B65" s="1" t="n"/>
       <c r="C65" s="1" t="n"/>
       <c r="D65" s="1" t="n"/>
@@ -2725,14 +2400,9 @@
       <c r="L65" s="4" t="n"/>
       <c r="M65" s="6" t="n"/>
       <c r="N65" s="6" t="n"/>
-      <c r="O65" s="4" t="n"/>
-      <c r="P65" s="4" t="n"/>
-      <c r="Q65" s="5" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>64</v>
-      </c>
+      <c r="A66" s="1" t="n"/>
       <c r="B66" s="1" t="n"/>
       <c r="C66" s="1" t="n"/>
       <c r="D66" s="1" t="n"/>
@@ -2746,14 +2416,9 @@
       <c r="L66" s="4" t="n"/>
       <c r="M66" s="6" t="n"/>
       <c r="N66" s="6" t="n"/>
-      <c r="O66" s="4" t="n"/>
-      <c r="P66" s="4" t="n"/>
-      <c r="Q66" s="5" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>65</v>
-      </c>
+      <c r="A67" s="1" t="n"/>
       <c r="B67" s="1" t="n"/>
       <c r="C67" s="1" t="n"/>
       <c r="D67" s="1" t="n"/>
@@ -2767,14 +2432,9 @@
       <c r="L67" s="4" t="n"/>
       <c r="M67" s="6" t="n"/>
       <c r="N67" s="6" t="n"/>
-      <c r="O67" s="4" t="n"/>
-      <c r="P67" s="4" t="n"/>
-      <c r="Q67" s="5" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>66</v>
-      </c>
+      <c r="A68" s="1" t="n"/>
       <c r="B68" s="1" t="n"/>
       <c r="C68" s="1" t="n"/>
       <c r="D68" s="1" t="n"/>
@@ -2788,14 +2448,9 @@
       <c r="L68" s="4" t="n"/>
       <c r="M68" s="6" t="n"/>
       <c r="N68" s="6" t="n"/>
-      <c r="O68" s="4" t="n"/>
-      <c r="P68" s="4" t="n"/>
-      <c r="Q68" s="5" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>67</v>
-      </c>
+      <c r="A69" s="1" t="n"/>
       <c r="B69" s="1" t="n"/>
       <c r="C69" s="1" t="n"/>
       <c r="D69" s="1" t="n"/>
@@ -2809,14 +2464,9 @@
       <c r="L69" s="4" t="n"/>
       <c r="M69" s="6" t="n"/>
       <c r="N69" s="6" t="n"/>
-      <c r="O69" s="4" t="n"/>
-      <c r="P69" s="4" t="n"/>
-      <c r="Q69" s="5" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>68</v>
-      </c>
+      <c r="A70" s="1" t="n"/>
       <c r="B70" s="1" t="n"/>
       <c r="C70" s="1" t="n"/>
       <c r="D70" s="1" t="n"/>
@@ -2830,14 +2480,9 @@
       <c r="L70" s="4" t="n"/>
       <c r="M70" s="6" t="n"/>
       <c r="N70" s="6" t="n"/>
-      <c r="O70" s="4" t="n"/>
-      <c r="P70" s="4" t="n"/>
-      <c r="Q70" s="5" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>69</v>
-      </c>
+      <c r="A71" s="1" t="n"/>
       <c r="B71" s="1" t="n"/>
       <c r="C71" s="1" t="n"/>
       <c r="D71" s="1" t="n"/>
@@ -2851,14 +2496,9 @@
       <c r="L71" s="4" t="n"/>
       <c r="M71" s="6" t="n"/>
       <c r="N71" s="6" t="n"/>
-      <c r="O71" s="4" t="n"/>
-      <c r="P71" s="4" t="n"/>
-      <c r="Q71" s="5" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>70</v>
-      </c>
+      <c r="A72" s="1" t="n"/>
       <c r="B72" s="1" t="n"/>
       <c r="C72" s="1" t="n"/>
       <c r="D72" s="1" t="n"/>
@@ -2872,14 +2512,9 @@
       <c r="L72" s="4" t="n"/>
       <c r="M72" s="6" t="n"/>
       <c r="N72" s="6" t="n"/>
-      <c r="O72" s="4" t="n"/>
-      <c r="P72" s="4" t="n"/>
-      <c r="Q72" s="5" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>71</v>
-      </c>
+      <c r="A73" s="1" t="n"/>
       <c r="B73" s="1" t="n"/>
       <c r="C73" s="1" t="n"/>
       <c r="D73" s="1" t="n"/>
@@ -2893,14 +2528,9 @@
       <c r="L73" s="4" t="n"/>
       <c r="M73" s="6" t="n"/>
       <c r="N73" s="6" t="n"/>
-      <c r="O73" s="4" t="n"/>
-      <c r="P73" s="4" t="n"/>
-      <c r="Q73" s="5" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>72</v>
-      </c>
+      <c r="A74" s="1" t="n"/>
       <c r="B74" s="1" t="n"/>
       <c r="C74" s="1" t="n"/>
       <c r="D74" s="1" t="n"/>
@@ -2914,14 +2544,9 @@
       <c r="L74" s="4" t="n"/>
       <c r="M74" s="6" t="n"/>
       <c r="N74" s="6" t="n"/>
-      <c r="O74" s="4" t="n"/>
-      <c r="P74" s="4" t="n"/>
-      <c r="Q74" s="5" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>73</v>
-      </c>
+      <c r="A75" s="1" t="n"/>
       <c r="B75" s="1" t="n"/>
       <c r="C75" s="1" t="n"/>
       <c r="D75" s="1" t="n"/>
@@ -2935,14 +2560,9 @@
       <c r="L75" s="4" t="n"/>
       <c r="M75" s="6" t="n"/>
       <c r="N75" s="6" t="n"/>
-      <c r="O75" s="4" t="n"/>
-      <c r="P75" s="4" t="n"/>
-      <c r="Q75" s="5" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
-        <v>74</v>
-      </c>
+      <c r="A76" s="1" t="n"/>
       <c r="B76" s="1" t="n"/>
       <c r="C76" s="1" t="n"/>
       <c r="D76" s="1" t="n"/>
@@ -2956,14 +2576,9 @@
       <c r="L76" s="4" t="n"/>
       <c r="M76" s="6" t="n"/>
       <c r="N76" s="6" t="n"/>
-      <c r="O76" s="4" t="n"/>
-      <c r="P76" s="4" t="n"/>
-      <c r="Q76" s="5" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
-        <v>75</v>
-      </c>
+      <c r="A77" s="1" t="n"/>
       <c r="B77" s="1" t="n"/>
       <c r="C77" s="1" t="n"/>
       <c r="D77" s="1" t="n"/>
@@ -2977,14 +2592,9 @@
       <c r="L77" s="4" t="n"/>
       <c r="M77" s="6" t="n"/>
       <c r="N77" s="6" t="n"/>
-      <c r="O77" s="4" t="n"/>
-      <c r="P77" s="4" t="n"/>
-      <c r="Q77" s="5" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
-        <v>76</v>
-      </c>
+      <c r="A78" s="1" t="n"/>
       <c r="B78" s="1" t="n"/>
       <c r="C78" s="1" t="n"/>
       <c r="D78" s="1" t="n"/>
@@ -2998,14 +2608,9 @@
       <c r="L78" s="4" t="n"/>
       <c r="M78" s="6" t="n"/>
       <c r="N78" s="6" t="n"/>
-      <c r="O78" s="4" t="n"/>
-      <c r="P78" s="4" t="n"/>
-      <c r="Q78" s="5" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
-        <v>77</v>
-      </c>
+      <c r="A79" s="1" t="n"/>
       <c r="B79" s="1" t="n"/>
       <c r="C79" s="1" t="n"/>
       <c r="D79" s="1" t="n"/>
@@ -3019,14 +2624,9 @@
       <c r="L79" s="4" t="n"/>
       <c r="M79" s="6" t="n"/>
       <c r="N79" s="6" t="n"/>
-      <c r="O79" s="4" t="n"/>
-      <c r="P79" s="4" t="n"/>
-      <c r="Q79" s="5" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
-        <v>78</v>
-      </c>
+      <c r="A80" s="1" t="n"/>
       <c r="B80" s="1" t="n"/>
       <c r="C80" s="1" t="n"/>
       <c r="D80" s="1" t="n"/>
@@ -3040,14 +2640,9 @@
       <c r="L80" s="4" t="n"/>
       <c r="M80" s="6" t="n"/>
       <c r="N80" s="6" t="n"/>
-      <c r="O80" s="4" t="n"/>
-      <c r="P80" s="4" t="n"/>
-      <c r="Q80" s="5" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
-        <v>79</v>
-      </c>
+      <c r="A81" s="1" t="n"/>
       <c r="B81" s="1" t="n"/>
       <c r="C81" s="1" t="n"/>
       <c r="D81" s="1" t="n"/>
@@ -3061,14 +2656,9 @@
       <c r="L81" s="4" t="n"/>
       <c r="M81" s="6" t="n"/>
       <c r="N81" s="6" t="n"/>
-      <c r="O81" s="4" t="n"/>
-      <c r="P81" s="4" t="n"/>
-      <c r="Q81" s="5" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
-        <v>80</v>
-      </c>
+      <c r="A82" s="1" t="n"/>
       <c r="B82" s="1" t="n"/>
       <c r="C82" s="1" t="n"/>
       <c r="D82" s="1" t="n"/>
@@ -3082,14 +2672,9 @@
       <c r="L82" s="4" t="n"/>
       <c r="M82" s="6" t="n"/>
       <c r="N82" s="6" t="n"/>
-      <c r="O82" s="4" t="n"/>
-      <c r="P82" s="4" t="n"/>
-      <c r="Q82" s="5" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
-        <v>81</v>
-      </c>
+      <c r="A83" s="1" t="n"/>
       <c r="B83" s="1" t="n"/>
       <c r="C83" s="1" t="n"/>
       <c r="D83" s="1" t="n"/>
@@ -3103,14 +2688,9 @@
       <c r="L83" s="4" t="n"/>
       <c r="M83" s="6" t="n"/>
       <c r="N83" s="6" t="n"/>
-      <c r="O83" s="4" t="n"/>
-      <c r="P83" s="4" t="n"/>
-      <c r="Q83" s="5" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
-        <v>82</v>
-      </c>
+      <c r="A84" s="1" t="n"/>
       <c r="B84" s="1" t="n"/>
       <c r="C84" s="1" t="n"/>
       <c r="D84" s="1" t="n"/>
@@ -3124,15 +2704,9 @@
       <c r="L84" s="4" t="n"/>
       <c r="M84" s="6" t="n"/>
       <c r="N84" s="6" t="n"/>
-      <c r="O84" s="4" t="n"/>
-      <c r="P84" s="4" t="n"/>
-      <c r="Q84" s="5" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="1">
-        <f>IF(E85="","",A84+1)</f>
-        <v/>
-      </c>
+      <c r="A85" s="1" t="n"/>
       <c r="B85" s="1" t="n"/>
       <c r="C85" s="1" t="n"/>
       <c r="D85" s="1" t="n"/>
@@ -3146,15 +2720,9 @@
       <c r="L85" s="4" t="n"/>
       <c r="M85" s="6" t="n"/>
       <c r="N85" s="6" t="n"/>
-      <c r="O85" s="4" t="n"/>
-      <c r="P85" s="4" t="n"/>
-      <c r="Q85" s="5" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="1">
-        <f>IF(E86="","",A85+1)</f>
-        <v/>
-      </c>
+      <c r="A86" s="1" t="n"/>
       <c r="B86" s="1" t="n"/>
       <c r="C86" s="1" t="n"/>
       <c r="D86" s="1" t="n"/>
@@ -3168,15 +2736,9 @@
       <c r="L86" s="4" t="n"/>
       <c r="M86" s="6" t="n"/>
       <c r="N86" s="6" t="n"/>
-      <c r="O86" s="4" t="n"/>
-      <c r="P86" s="4" t="n"/>
-      <c r="Q86" s="5" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="1">
-        <f>IF(E87="","",A86+1)</f>
-        <v/>
-      </c>
+      <c r="A87" s="1" t="n"/>
       <c r="B87" s="1" t="n"/>
       <c r="C87" s="1" t="n"/>
       <c r="D87" s="1" t="n"/>
@@ -3190,15 +2752,9 @@
       <c r="L87" s="4" t="n"/>
       <c r="M87" s="6" t="n"/>
       <c r="N87" s="6" t="n"/>
-      <c r="O87" s="4" t="n"/>
-      <c r="P87" s="4" t="n"/>
-      <c r="Q87" s="5" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="1">
-        <f>IF(E88="","",A87+1)</f>
-        <v/>
-      </c>
+      <c r="A88" s="1" t="n"/>
       <c r="B88" s="1" t="n"/>
       <c r="C88" s="1" t="n"/>
       <c r="D88" s="1" t="n"/>
@@ -3212,15 +2768,9 @@
       <c r="L88" s="4" t="n"/>
       <c r="M88" s="6" t="n"/>
       <c r="N88" s="6" t="n"/>
-      <c r="O88" s="4" t="n"/>
-      <c r="P88" s="4" t="n"/>
-      <c r="Q88" s="5" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="1">
-        <f>IF(E89="","",A88+1)</f>
-        <v/>
-      </c>
+      <c r="A89" s="1" t="n"/>
       <c r="B89" s="1" t="n"/>
       <c r="C89" s="1" t="n"/>
       <c r="D89" s="1" t="n"/>
@@ -3234,15 +2784,9 @@
       <c r="L89" s="4" t="n"/>
       <c r="M89" s="6" t="n"/>
       <c r="N89" s="6" t="n"/>
-      <c r="O89" s="4" t="n"/>
-      <c r="P89" s="4" t="n"/>
-      <c r="Q89" s="5" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="1">
-        <f>IF(E90="","",A89+1)</f>
-        <v/>
-      </c>
+      <c r="A90" s="1" t="n"/>
       <c r="B90" s="1" t="n"/>
       <c r="C90" s="1" t="n"/>
       <c r="D90" s="1" t="n"/>
@@ -3256,15 +2800,9 @@
       <c r="L90" s="4" t="n"/>
       <c r="M90" s="6" t="n"/>
       <c r="N90" s="6" t="n"/>
-      <c r="O90" s="4" t="n"/>
-      <c r="P90" s="4" t="n"/>
-      <c r="Q90" s="5" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="1">
-        <f>IF(E91="","",A90+1)</f>
-        <v/>
-      </c>
+      <c r="A91" s="1" t="n"/>
       <c r="B91" s="1" t="n"/>
       <c r="C91" s="1" t="n"/>
       <c r="D91" s="1" t="n"/>
@@ -3278,15 +2816,9 @@
       <c r="L91" s="4" t="n"/>
       <c r="M91" s="6" t="n"/>
       <c r="N91" s="6" t="n"/>
-      <c r="O91" s="4" t="n"/>
-      <c r="P91" s="4" t="n"/>
-      <c r="Q91" s="5" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="1">
-        <f>IF(E92="","",A91+1)</f>
-        <v/>
-      </c>
+      <c r="A92" s="1" t="n"/>
       <c r="B92" s="1" t="n"/>
       <c r="C92" s="1" t="n"/>
       <c r="D92" s="1" t="n"/>
@@ -3300,15 +2832,9 @@
       <c r="L92" s="4" t="n"/>
       <c r="M92" s="6" t="n"/>
       <c r="N92" s="6" t="n"/>
-      <c r="O92" s="4" t="n"/>
-      <c r="P92" s="4" t="n"/>
-      <c r="Q92" s="5" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="1">
-        <f>IF(E93="","",A92+1)</f>
-        <v/>
-      </c>
+      <c r="A93" s="1" t="n"/>
       <c r="B93" s="1" t="n"/>
       <c r="C93" s="1" t="n"/>
       <c r="D93" s="1" t="n"/>
@@ -3322,15 +2848,9 @@
       <c r="L93" s="4" t="n"/>
       <c r="M93" s="6" t="n"/>
       <c r="N93" s="6" t="n"/>
-      <c r="O93" s="4" t="n"/>
-      <c r="P93" s="4" t="n"/>
-      <c r="Q93" s="5" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="1">
-        <f>IF(E94="","",A93+1)</f>
-        <v/>
-      </c>
+      <c r="A94" s="1" t="n"/>
       <c r="B94" s="1" t="n"/>
       <c r="C94" s="1" t="n"/>
       <c r="D94" s="1" t="n"/>
@@ -3344,15 +2864,9 @@
       <c r="L94" s="4" t="n"/>
       <c r="M94" s="6" t="n"/>
       <c r="N94" s="6" t="n"/>
-      <c r="O94" s="4" t="n"/>
-      <c r="P94" s="4" t="n"/>
-      <c r="Q94" s="5" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="1">
-        <f>IF(E95="","",A94+1)</f>
-        <v/>
-      </c>
+      <c r="A95" s="1" t="n"/>
       <c r="B95" s="1" t="n"/>
       <c r="C95" s="1" t="n"/>
       <c r="D95" s="1" t="n"/>
@@ -3366,15 +2880,9 @@
       <c r="L95" s="4" t="n"/>
       <c r="M95" s="6" t="n"/>
       <c r="N95" s="6" t="n"/>
-      <c r="O95" s="4" t="n"/>
-      <c r="P95" s="4" t="n"/>
-      <c r="Q95" s="5" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="1">
-        <f>IF(E96="","",A95+1)</f>
-        <v/>
-      </c>
+      <c r="A96" s="1" t="n"/>
       <c r="B96" s="1" t="n"/>
       <c r="C96" s="1" t="n"/>
       <c r="D96" s="1" t="n"/>
@@ -3388,15 +2896,9 @@
       <c r="L96" s="4" t="n"/>
       <c r="M96" s="6" t="n"/>
       <c r="N96" s="6" t="n"/>
-      <c r="O96" s="4" t="n"/>
-      <c r="P96" s="4" t="n"/>
-      <c r="Q96" s="5" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="1">
-        <f>IF(E97="","",A96+1)</f>
-        <v/>
-      </c>
+      <c r="A97" s="1" t="n"/>
       <c r="B97" s="1" t="n"/>
       <c r="C97" s="1" t="n"/>
       <c r="D97" s="1" t="n"/>
@@ -3410,15 +2912,9 @@
       <c r="L97" s="4" t="n"/>
       <c r="M97" s="6" t="n"/>
       <c r="N97" s="6" t="n"/>
-      <c r="O97" s="4" t="n"/>
-      <c r="P97" s="4" t="n"/>
-      <c r="Q97" s="5" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="1">
-        <f>IF(E98="","",A97+1)</f>
-        <v/>
-      </c>
+      <c r="A98" s="1" t="n"/>
       <c r="B98" s="1" t="n"/>
       <c r="C98" s="1" t="n"/>
       <c r="D98" s="1" t="n"/>
@@ -3432,15 +2928,9 @@
       <c r="L98" s="4" t="n"/>
       <c r="M98" s="6" t="n"/>
       <c r="N98" s="6" t="n"/>
-      <c r="O98" s="4" t="n"/>
-      <c r="P98" s="4" t="n"/>
-      <c r="Q98" s="5" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="1">
-        <f>IF(E99="","",A98+1)</f>
-        <v/>
-      </c>
+      <c r="A99" s="1" t="n"/>
       <c r="B99" s="1" t="n"/>
       <c r="C99" s="1" t="n"/>
       <c r="D99" s="1" t="n"/>
@@ -3454,15 +2944,9 @@
       <c r="L99" s="4" t="n"/>
       <c r="M99" s="6" t="n"/>
       <c r="N99" s="6" t="n"/>
-      <c r="O99" s="4" t="n"/>
-      <c r="P99" s="4" t="n"/>
-      <c r="Q99" s="5" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="1">
-        <f>IF(E100="","",A99+1)</f>
-        <v/>
-      </c>
+      <c r="A100" s="1" t="n"/>
       <c r="B100" s="1" t="n"/>
       <c r="C100" s="1" t="n"/>
       <c r="D100" s="1" t="n"/>
@@ -3476,15 +2960,9 @@
       <c r="L100" s="4" t="n"/>
       <c r="M100" s="6" t="n"/>
       <c r="N100" s="6" t="n"/>
-      <c r="O100" s="4" t="n"/>
-      <c r="P100" s="4" t="n"/>
-      <c r="Q100" s="5" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="1">
-        <f>IF(E101="","",A100+1)</f>
-        <v/>
-      </c>
+      <c r="A101" s="1" t="n"/>
       <c r="B101" s="1" t="n"/>
       <c r="C101" s="1" t="n"/>
       <c r="D101" s="1" t="n"/>
@@ -3498,15 +2976,9 @@
       <c r="L101" s="4" t="n"/>
       <c r="M101" s="6" t="n"/>
       <c r="N101" s="6" t="n"/>
-      <c r="O101" s="4" t="n"/>
-      <c r="P101" s="4" t="n"/>
-      <c r="Q101" s="5" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="1">
-        <f>IF(E102="","",A101+1)</f>
-        <v/>
-      </c>
+      <c r="A102" s="1" t="n"/>
       <c r="B102" s="1" t="n"/>
       <c r="C102" s="1" t="n"/>
       <c r="D102" s="1" t="n"/>
@@ -3520,15 +2992,9 @@
       <c r="L102" s="4" t="n"/>
       <c r="M102" s="6" t="n"/>
       <c r="N102" s="6" t="n"/>
-      <c r="O102" s="4" t="n"/>
-      <c r="P102" s="4" t="n"/>
-      <c r="Q102" s="5" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="1">
-        <f>IF(E103="","",A102+1)</f>
-        <v/>
-      </c>
+      <c r="A103" s="1" t="n"/>
       <c r="B103" s="1" t="n"/>
       <c r="C103" s="1" t="n"/>
       <c r="D103" s="1" t="n"/>
@@ -3542,15 +3008,9 @@
       <c r="L103" s="4" t="n"/>
       <c r="M103" s="6" t="n"/>
       <c r="N103" s="6" t="n"/>
-      <c r="O103" s="4" t="n"/>
-      <c r="P103" s="4" t="n"/>
-      <c r="Q103" s="5" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="1">
-        <f>IF(E104="","",A103+1)</f>
-        <v/>
-      </c>
+      <c r="A104" s="1" t="n"/>
       <c r="B104" s="1" t="n"/>
       <c r="C104" s="1" t="n"/>
       <c r="D104" s="1" t="n"/>
@@ -3564,15 +3024,9 @@
       <c r="L104" s="4" t="n"/>
       <c r="M104" s="6" t="n"/>
       <c r="N104" s="6" t="n"/>
-      <c r="O104" s="4" t="n"/>
-      <c r="P104" s="4" t="n"/>
-      <c r="Q104" s="5" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="1">
-        <f>IF(E105="","",A104+1)</f>
-        <v/>
-      </c>
+      <c r="A105" s="1" t="n"/>
       <c r="B105" s="1" t="n"/>
       <c r="C105" s="1" t="n"/>
       <c r="D105" s="1" t="n"/>
@@ -3586,15 +3040,9 @@
       <c r="L105" s="4" t="n"/>
       <c r="M105" s="6" t="n"/>
       <c r="N105" s="6" t="n"/>
-      <c r="O105" s="4" t="n"/>
-      <c r="P105" s="4" t="n"/>
-      <c r="Q105" s="5" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="1">
-        <f>IF(E106="","",A105+1)</f>
-        <v/>
-      </c>
+      <c r="A106" s="1" t="n"/>
       <c r="B106" s="1" t="n"/>
       <c r="C106" s="1" t="n"/>
       <c r="D106" s="1" t="n"/>
@@ -3608,15 +3056,9 @@
       <c r="L106" s="4" t="n"/>
       <c r="M106" s="6" t="n"/>
       <c r="N106" s="6" t="n"/>
-      <c r="O106" s="4" t="n"/>
-      <c r="P106" s="4" t="n"/>
-      <c r="Q106" s="5" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="1">
-        <f>IF(E107="","",A106+1)</f>
-        <v/>
-      </c>
+      <c r="A107" s="1" t="n"/>
       <c r="B107" s="1" t="n"/>
       <c r="C107" s="1" t="n"/>
       <c r="D107" s="1" t="n"/>
@@ -3630,15 +3072,9 @@
       <c r="L107" s="4" t="n"/>
       <c r="M107" s="6" t="n"/>
       <c r="N107" s="6" t="n"/>
-      <c r="O107" s="4" t="n"/>
-      <c r="P107" s="4" t="n"/>
-      <c r="Q107" s="5" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="1">
-        <f>IF(E108="","",A107+1)</f>
-        <v/>
-      </c>
+      <c r="A108" s="1" t="n"/>
       <c r="B108" s="1" t="n"/>
       <c r="C108" s="1" t="n"/>
       <c r="D108" s="1" t="n"/>
@@ -3652,15 +3088,9 @@
       <c r="L108" s="4" t="n"/>
       <c r="M108" s="6" t="n"/>
       <c r="N108" s="6" t="n"/>
-      <c r="O108" s="4" t="n"/>
-      <c r="P108" s="4" t="n"/>
-      <c r="Q108" s="5" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="1">
-        <f>IF(E109="","",A108+1)</f>
-        <v/>
-      </c>
+      <c r="A109" s="1" t="n"/>
       <c r="B109" s="1" t="n"/>
       <c r="C109" s="1" t="n"/>
       <c r="D109" s="1" t="n"/>
@@ -3674,15 +3104,9 @@
       <c r="L109" s="4" t="n"/>
       <c r="M109" s="6" t="n"/>
       <c r="N109" s="6" t="n"/>
-      <c r="O109" s="4" t="n"/>
-      <c r="P109" s="4" t="n"/>
-      <c r="Q109" s="5" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="1">
-        <f>IF(E110="","",A109+1)</f>
-        <v/>
-      </c>
+      <c r="A110" s="1" t="n"/>
       <c r="B110" s="1" t="n"/>
       <c r="C110" s="1" t="n"/>
       <c r="D110" s="1" t="n"/>
@@ -3696,15 +3120,9 @@
       <c r="L110" s="4" t="n"/>
       <c r="M110" s="6" t="n"/>
       <c r="N110" s="6" t="n"/>
-      <c r="O110" s="4" t="n"/>
-      <c r="P110" s="4" t="n"/>
-      <c r="Q110" s="5" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="1">
-        <f>IF(E111="","",A110+1)</f>
-        <v/>
-      </c>
+      <c r="A111" s="1" t="n"/>
       <c r="B111" s="1" t="n"/>
       <c r="C111" s="1" t="n"/>
       <c r="D111" s="1" t="n"/>
@@ -3718,15 +3136,9 @@
       <c r="L111" s="4" t="n"/>
       <c r="M111" s="6" t="n"/>
       <c r="N111" s="6" t="n"/>
-      <c r="O111" s="4" t="n"/>
-      <c r="P111" s="4" t="n"/>
-      <c r="Q111" s="5" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="1">
-        <f>IF(E112="","",A111+1)</f>
-        <v/>
-      </c>
+      <c r="A112" s="1" t="n"/>
       <c r="B112" s="1" t="n"/>
       <c r="C112" s="1" t="n"/>
       <c r="D112" s="1" t="n"/>
@@ -3740,15 +3152,9 @@
       <c r="L112" s="4" t="n"/>
       <c r="M112" s="6" t="n"/>
       <c r="N112" s="6" t="n"/>
-      <c r="O112" s="4" t="n"/>
-      <c r="P112" s="4" t="n"/>
-      <c r="Q112" s="5" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="1">
-        <f>IF(E113="","",A112+1)</f>
-        <v/>
-      </c>
+      <c r="A113" s="1" t="n"/>
       <c r="B113" s="1" t="n"/>
       <c r="C113" s="1" t="n"/>
       <c r="D113" s="1" t="n"/>
@@ -3762,15 +3168,9 @@
       <c r="L113" s="4" t="n"/>
       <c r="M113" s="6" t="n"/>
       <c r="N113" s="6" t="n"/>
-      <c r="O113" s="4" t="n"/>
-      <c r="P113" s="4" t="n"/>
-      <c r="Q113" s="5" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="1">
-        <f>IF(E114="","",A113+1)</f>
-        <v/>
-      </c>
+      <c r="A114" s="1" t="n"/>
       <c r="B114" s="1" t="n"/>
       <c r="C114" s="1" t="n"/>
       <c r="D114" s="1" t="n"/>
@@ -3784,15 +3184,9 @@
       <c r="L114" s="4" t="n"/>
       <c r="M114" s="6" t="n"/>
       <c r="N114" s="6" t="n"/>
-      <c r="O114" s="4" t="n"/>
-      <c r="P114" s="4" t="n"/>
-      <c r="Q114" s="5" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="1">
-        <f>IF(E115="","",A114+1)</f>
-        <v/>
-      </c>
+      <c r="A115" s="1" t="n"/>
       <c r="B115" s="1" t="n"/>
       <c r="C115" s="1" t="n"/>
       <c r="D115" s="1" t="n"/>
@@ -3806,15 +3200,9 @@
       <c r="L115" s="4" t="n"/>
       <c r="M115" s="6" t="n"/>
       <c r="N115" s="6" t="n"/>
-      <c r="O115" s="4" t="n"/>
-      <c r="P115" s="4" t="n"/>
-      <c r="Q115" s="5" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="1">
-        <f>IF(E116="","",A115+1)</f>
-        <v/>
-      </c>
+      <c r="A116" s="1" t="n"/>
       <c r="B116" s="1" t="n"/>
       <c r="C116" s="1" t="n"/>
       <c r="D116" s="1" t="n"/>
@@ -3828,15 +3216,9 @@
       <c r="L116" s="4" t="n"/>
       <c r="M116" s="6" t="n"/>
       <c r="N116" s="6" t="n"/>
-      <c r="O116" s="4" t="n"/>
-      <c r="P116" s="4" t="n"/>
-      <c r="Q116" s="5" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="1">
-        <f>IF(E117="","",A116+1)</f>
-        <v/>
-      </c>
+      <c r="A117" s="1" t="n"/>
       <c r="B117" s="1" t="n"/>
       <c r="C117" s="1" t="n"/>
       <c r="D117" s="1" t="n"/>
@@ -3850,15 +3232,9 @@
       <c r="L117" s="4" t="n"/>
       <c r="M117" s="6" t="n"/>
       <c r="N117" s="6" t="n"/>
-      <c r="O117" s="4" t="n"/>
-      <c r="P117" s="4" t="n"/>
-      <c r="Q117" s="5" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="1">
-        <f>IF(E118="","",A117+1)</f>
-        <v/>
-      </c>
+      <c r="A118" s="1" t="n"/>
       <c r="B118" s="1" t="n"/>
       <c r="C118" s="1" t="n"/>
       <c r="D118" s="1" t="n"/>
@@ -3872,15 +3248,9 @@
       <c r="L118" s="4" t="n"/>
       <c r="M118" s="6" t="n"/>
       <c r="N118" s="6" t="n"/>
-      <c r="O118" s="4" t="n"/>
-      <c r="P118" s="4" t="n"/>
-      <c r="Q118" s="5" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="1">
-        <f>IF(E119="","",A118+1)</f>
-        <v/>
-      </c>
+      <c r="A119" s="1" t="n"/>
       <c r="B119" s="1" t="n"/>
       <c r="C119" s="1" t="n"/>
       <c r="D119" s="1" t="n"/>
@@ -3892,15 +3262,9 @@
       <c r="J119" s="3" t="n"/>
       <c r="K119" s="4" t="n"/>
       <c r="L119" s="4" t="n"/>
-      <c r="O119" s="4" t="n"/>
-      <c r="P119" s="4" t="n"/>
-      <c r="Q119" s="5" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="1">
-        <f>IF(E120="","",A119+1)</f>
-        <v/>
-      </c>
+      <c r="A120" s="1" t="n"/>
       <c r="B120" s="1" t="n"/>
       <c r="C120" s="1" t="n"/>
       <c r="D120" s="1" t="n"/>
@@ -3912,15 +3276,9 @@
       <c r="J120" s="3" t="n"/>
       <c r="K120" s="4" t="n"/>
       <c r="L120" s="4" t="n"/>
-      <c r="O120" s="4" t="n"/>
-      <c r="P120" s="4" t="n"/>
-      <c r="Q120" s="5" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="1">
-        <f>IF(E121="","",A120+1)</f>
-        <v/>
-      </c>
+      <c r="A121" s="1" t="n"/>
       <c r="B121" s="1" t="n"/>
       <c r="C121" s="1" t="n"/>
       <c r="D121" s="1" t="n"/>
@@ -3932,15 +3290,9 @@
       <c r="J121" s="3" t="n"/>
       <c r="K121" s="4" t="n"/>
       <c r="L121" s="4" t="n"/>
-      <c r="O121" s="4" t="n"/>
-      <c r="P121" s="4" t="n"/>
-      <c r="Q121" s="5" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="1">
-        <f>IF(E122="","",A121+1)</f>
-        <v/>
-      </c>
+      <c r="A122" s="1" t="n"/>
       <c r="B122" s="1" t="n"/>
       <c r="C122" s="1" t="n"/>
       <c r="D122" s="1" t="n"/>
@@ -3952,9 +3304,6 @@
       <c r="J122" s="3" t="n"/>
       <c r="K122" s="4" t="n"/>
       <c r="L122" s="4" t="n"/>
-      <c r="O122" s="4" t="n"/>
-      <c r="P122" s="4" t="n"/>
-      <c r="Q122" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Stephen: Kranz Paychex access granted — add to collection
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_2026-09-25.xlsx
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O122"/>
+  <dimension ref="A2:O122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -704,7 +704,6 @@
     <col width="38" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="74.45" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
@@ -1022,11 +1021,7 @@
         <v/>
       </c>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="45" t="inlineStr">
-        <is>
-          <t>No access — client has not granted it</t>
-        </is>
-      </c>
+      <c r="O6" s="45" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">

</xml_diff>